<commit_message>
excel file updated and add new Word file
</commit_message>
<xml_diff>
--- a/Ah.xlsx
+++ b/Ah.xlsx
@@ -16,6 +16,23 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>ahmed</t>
+  </si>
+  <si>
+    <t>mohamed</t>
+  </si>
+  <si>
+    <t>Names</t>
+  </si>
+  <si>
+    <t>Salary</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -49,8 +66,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -331,9 +351,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2000</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>